<commit_message>
updated seleniu code on homepage categories section ecommerse
</commit_message>
<xml_diff>
--- a/ecommerse_automation_maven_gurupreeth/project_documents.xlsx
+++ b/ecommerse_automation_maven_gurupreeth/project_documents.xlsx
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="65">
   <si>
     <t>title</t>
   </si>
@@ -228,6 +228,24 @@
   </si>
   <si>
     <t>http://localhost:5173/</t>
+  </si>
+  <si>
+    <t>category main heading text</t>
+  </si>
+  <si>
+    <t>Explore Categories</t>
+  </si>
+  <si>
+    <t>Category sub heading text</t>
+  </si>
+  <si>
+    <t>Tap any category to instantly search products.</t>
+  </si>
+  <si>
+    <t>Category count text</t>
+  </si>
+  <si>
+    <t>Showing 7 of 10 categories</t>
   </si>
 </sst>
 </file>
@@ -549,7 +567,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -557,24 +575,37 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.28515625" customWidth="1"/>
-    <col min="2" max="2" width="21.7109375" customWidth="1"/>
-    <col min="3" max="3" width="28.5703125" customWidth="1"/>
-    <col min="4" max="4" width="37" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5">
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="42.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="F1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -590,13 +621,22 @@
       <c r="E2">
         <v>12345</v>
       </c>
-    </row>
-    <row r="4" spans="1:5">
+      <c r="F2" t="s">
+        <v>60</v>
+      </c>
+      <c r="G2" t="s">
+        <v>62</v>
+      </c>
+      <c r="H2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="D4" s="2">
         <v>49290</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:8">
       <c r="A6" t="s">
         <v>21</v>
       </c>

</xml_diff>

<commit_message>
regression scenarios on category, Footer regression scenario
</commit_message>
<xml_diff>
--- a/ecommerse_automation_maven_gurupreeth/project_documents.xlsx
+++ b/ecommerse_automation_maven_gurupreeth/project_documents.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="6" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="916"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="916" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Homepage" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="400">
   <si>
     <t>title</t>
   </si>
@@ -639,13 +639,650 @@
   </si>
   <si>
     <t>Office Supplies</t>
+  </si>
+  <si>
+    <t>plainaddress</t>
+  </si>
+  <si>
+    <t>user.domain.com</t>
+  </si>
+  <si>
+    <t>userdomaincom</t>
+  </si>
+  <si>
+    <t>helloworld</t>
+  </si>
+  <si>
+    <t>test-at-gmail-dot-com</t>
+  </si>
+  <si>
+    <t>abc.gmail.com</t>
+  </si>
+  <si>
+    <t>abcgmailcom</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>username.domain.co.in</t>
+  </si>
+  <si>
+    <t>@gmail.com</t>
+  </si>
+  <si>
+    <t>@example.org</t>
+  </si>
+  <si>
+    <t>@domain.com</t>
+  </si>
+  <si>
+    <t>@domain.co.in</t>
+  </si>
+  <si>
+    <t>@.com</t>
+  </si>
+  <si>
+    <t>@.domain.com</t>
+  </si>
+  <si>
+    <t>abc@</t>
+  </si>
+  <si>
+    <t>user@</t>
+  </si>
+  <si>
+    <t>test@</t>
+  </si>
+  <si>
+    <t>abc123@</t>
+  </si>
+  <si>
+    <t>abc@gmail</t>
+  </si>
+  <si>
+    <t>user@domain</t>
+  </si>
+  <si>
+    <t>name@company</t>
+  </si>
+  <si>
+    <t>test@localhost</t>
+  </si>
+  <si>
+    <t>abc@subdomain</t>
+  </si>
+  <si>
+    <t>abc@.com</t>
+  </si>
+  <si>
+    <t>abc@.gmail.com</t>
+  </si>
+  <si>
+    <t>abc@.domain.com</t>
+  </si>
+  <si>
+    <t>abc@.domain.co.in</t>
+  </si>
+  <si>
+    <t>abc@com.</t>
+  </si>
+  <si>
+    <t>abc@gmail.</t>
+  </si>
+  <si>
+    <t>abc@domain.</t>
+  </si>
+  <si>
+    <t>abc@domain.co.</t>
+  </si>
+  <si>
+    <t>abc..def@gmail.com</t>
+  </si>
+  <si>
+    <t>abc...def@gmail.com</t>
+  </si>
+  <si>
+    <t>abc..@gmail.com</t>
+  </si>
+  <si>
+    <t>..abc@gmail.com</t>
+  </si>
+  <si>
+    <t>abc@domain..com</t>
+  </si>
+  <si>
+    <t>abc@domain...com</t>
+  </si>
+  <si>
+    <t>abc@sub..domain.com</t>
+  </si>
+  <si>
+    <t>abc@sub.domain..com</t>
+  </si>
+  <si>
+    <t>abc@gmail..co.in</t>
+  </si>
+  <si>
+    <t>abc@domain..co.in</t>
+  </si>
+  <si>
+    <t>abc@domain..</t>
+  </si>
+  <si>
+    <t>abc@..domain.com</t>
+  </si>
+  <si>
+    <t>abc@.gmail..com</t>
+  </si>
+  <si>
+    <t>a@b@c.com</t>
+  </si>
+  <si>
+    <t>user@@gmail.com</t>
+  </si>
+  <si>
+    <t>abc@domain@com</t>
+  </si>
+  <si>
+    <t>abc@@domain.com</t>
+  </si>
+  <si>
+    <t>a@@b@@c.com</t>
+  </si>
+  <si>
+    <t>a bc@gmail.com</t>
+  </si>
+  <si>
+    <t>ab c@domain.com</t>
+  </si>
+  <si>
+    <t>abc @gmail.com</t>
+  </si>
+  <si>
+    <t>abc@ gmail.com</t>
+  </si>
+  <si>
+    <t>abc@gmail .com</t>
+  </si>
+  <si>
+    <t>abc@domain .com</t>
+  </si>
+  <si>
+    <t>abc@ domain.com</t>
+  </si>
+  <si>
+    <t>abc@gmail.com</t>
+  </si>
+  <si>
+    <t>abc#gmail.com</t>
+  </si>
+  <si>
+    <t>abc!gmail.com</t>
+  </si>
+  <si>
+    <t>abc$gmail.com</t>
+  </si>
+  <si>
+    <t>abc%gmail.com</t>
+  </si>
+  <si>
+    <t>abc^gmail.com</t>
+  </si>
+  <si>
+    <t>abc&amp;gmail.com</t>
+  </si>
+  <si>
+    <r>
+      <t>abc</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>gmail.com</t>
+    </r>
+  </si>
+  <si>
+    <t>abc(gmail.com</t>
+  </si>
+  <si>
+    <t>abc)gmail.com</t>
+  </si>
+  <si>
+    <t>abc=gmail.com</t>
+  </si>
+  <si>
+    <t>abc+gmail.com</t>
+  </si>
+  <si>
+    <t>abc,gmail.com</t>
+  </si>
+  <si>
+    <t>abc;gmail.com</t>
+  </si>
+  <si>
+    <t>abc:gmail.com</t>
+  </si>
+  <si>
+    <t>abc/gmail.com</t>
+  </si>
+  <si>
+    <t>abc\gmail.com</t>
+  </si>
+  <si>
+    <t>abc|gmail.com</t>
+  </si>
+  <si>
+    <t>abc[gmail.com</t>
+  </si>
+  <si>
+    <t>abc]gmail.com</t>
+  </si>
+  <si>
+    <t>abc{gmail.com</t>
+  </si>
+  <si>
+    <t>abc}gmail.com</t>
+  </si>
+  <si>
+    <t>abc@domain#com</t>
+  </si>
+  <si>
+    <t>abc@domain!com</t>
+  </si>
+  <si>
+    <t>abc@domain$com</t>
+  </si>
+  <si>
+    <t>abc@domain%com</t>
+  </si>
+  <si>
+    <t>abc@domain^com</t>
+  </si>
+  <si>
+    <t>abc@domain&amp;com</t>
+  </si>
+  <si>
+    <r>
+      <t>abc@domain</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>com</t>
+    </r>
+  </si>
+  <si>
+    <t>abc@domain(com</t>
+  </si>
+  <si>
+    <t>abc@domain)com</t>
+  </si>
+  <si>
+    <t>abc@domain=com</t>
+  </si>
+  <si>
+    <t>abc@domain+com</t>
+  </si>
+  <si>
+    <t>abc@domain,com</t>
+  </si>
+  <si>
+    <t>abc@domain;com</t>
+  </si>
+  <si>
+    <t>abc@domain:com</t>
+  </si>
+  <si>
+    <t>abc@domain/com</t>
+  </si>
+  <si>
+    <t>abc@domain\com</t>
+  </si>
+  <si>
+    <t>abc@domain|com</t>
+  </si>
+  <si>
+    <t>abc@domain[com</t>
+  </si>
+  <si>
+    <t>abc@domain]com</t>
+  </si>
+  <si>
+    <t>abc@domain{com</t>
+  </si>
+  <si>
+    <t>abc@domain}com</t>
+  </si>
+  <si>
+    <t>.abc@gmail.com</t>
+  </si>
+  <si>
+    <t>abc.@gmail.com</t>
+  </si>
+  <si>
+    <t>.first.last@gmail.com</t>
+  </si>
+  <si>
+    <t>abc..last@gmail.com</t>
+  </si>
+  <si>
+    <t>abc@-domain.com</t>
+  </si>
+  <si>
+    <t>abc@domain-.com</t>
+  </si>
+  <si>
+    <t>abc@sub-domain-.com</t>
+  </si>
+  <si>
+    <t>abc@-subdomain.com</t>
+  </si>
+  <si>
+    <t>abc@domain_.com</t>
+  </si>
+  <si>
+    <t>abc@_domain.com</t>
+  </si>
+  <si>
+    <t>abc@sub_domain.com</t>
+  </si>
+  <si>
+    <t>abc@gmail/com</t>
+  </si>
+  <si>
+    <t>abc@gmail\com</t>
+  </si>
+  <si>
+    <t>abc@domain/co.in</t>
+  </si>
+  <si>
+    <t>abc@domain\co.in</t>
+  </si>
+  <si>
+    <t>abc@gmail,com</t>
+  </si>
+  <si>
+    <t>abc@domain,org</t>
+  </si>
+  <si>
+    <t>abc@domain,co.in</t>
+  </si>
+  <si>
+    <t>abc;def@gmail.com</t>
+  </si>
+  <si>
+    <t>abc:def@gmail.com</t>
+  </si>
+  <si>
+    <t>abc|def@gmail.com</t>
+  </si>
+  <si>
+    <t>abc@domain\tcom</t>
+  </si>
+  <si>
+    <t>abc\n@gmail.com</t>
+  </si>
+  <si>
+    <t>abc\r@gmail.com</t>
+  </si>
+  <si>
+    <t>abc\t@gmail.com</t>
+  </si>
+  <si>
+    <t>abc@domain.1</t>
+  </si>
+  <si>
+    <t>abc@domain.12</t>
+  </si>
+  <si>
+    <t>abc@domain.123</t>
+  </si>
+  <si>
+    <t>abc@domain.c1</t>
+  </si>
+  <si>
+    <t>abc@domain.1c</t>
+  </si>
+  <si>
+    <t>abc@gmail.c</t>
+  </si>
+  <si>
+    <t>user@domain.x</t>
+  </si>
+  <si>
+    <t>test@company.z</t>
+  </si>
+  <si>
+    <t>abc@111.222.333.44444</t>
+  </si>
+  <si>
+    <t>abc@999.999.999.999</t>
+  </si>
+  <si>
+    <t>abc@1.1.1</t>
+  </si>
+  <si>
+    <t>abc@256.256.256.256</t>
+  </si>
+  <si>
+    <t>@abc</t>
+  </si>
+  <si>
+    <t>@</t>
+  </si>
+  <si>
+    <t>abc@@</t>
+  </si>
+  <si>
+    <t>@@gmail.com</t>
+  </si>
+  <si>
+    <t>abc.@.gmail.com</t>
+  </si>
+  <si>
+    <t>abc@domain@</t>
+  </si>
+  <si>
+    <t>abc..@domain.com</t>
+  </si>
+  <si>
+    <t>abc@..com</t>
+  </si>
+  <si>
+    <t>abc@com..</t>
+  </si>
+  <si>
+    <t>abc@.</t>
+  </si>
+  <si>
+    <t>.@.</t>
+  </si>
+  <si>
+    <t>abc@domain#co.in</t>
+  </si>
+  <si>
+    <t>abc@domain!.co.in</t>
+  </si>
+  <si>
+    <t>abc@domain$.co.in</t>
+  </si>
+  <si>
+    <t>abc@domain..123</t>
+  </si>
+  <si>
+    <t>abc@domain.toolongtlddddddddddddd</t>
+  </si>
+  <si>
+    <t>hello world</t>
+  </si>
+  <si>
+    <t>my email is abc@gmail.com</t>
+  </si>
+  <si>
+    <t>gmail.com</t>
+  </si>
+  <si>
+    <t>justtext</t>
+  </si>
+  <si>
+    <t>notanemail</t>
+  </si>
+  <si>
+    <t>none</t>
+  </si>
+  <si>
+    <t>null</t>
+  </si>
+  <si>
+    <t>undefined</t>
+  </si>
+  <si>
+    <t xml:space="preserve">invalid email ids. </t>
+  </si>
+  <si>
+    <t>Valid email id</t>
+  </si>
+  <si>
+    <t>test@yahoo.com</t>
+  </si>
+  <si>
+    <t>user@outlook.com</t>
+  </si>
+  <si>
+    <t>hello@domain.com</t>
+  </si>
+  <si>
+    <t>sample@company.org</t>
+  </si>
+  <si>
+    <t>abc123@gmail.com</t>
+  </si>
+  <si>
+    <t>user2024@domain.com</t>
+  </si>
+  <si>
+    <t>test001@yahoo.in</t>
+  </si>
+  <si>
+    <t>123user@company.org</t>
+  </si>
+  <si>
+    <t>first.last@gmail.com</t>
+  </si>
+  <si>
+    <t>user.name@domain.com</t>
+  </si>
+  <si>
+    <t>a.b.c@gmail.com</t>
+  </si>
+  <si>
+    <t>firstname.lastname@company.org</t>
+  </si>
+  <si>
+    <t>user_name@gmail.com</t>
+  </si>
+  <si>
+    <t>test_user@domain.com</t>
+  </si>
+  <si>
+    <t>first_last@company.co.in</t>
+  </si>
+  <si>
+    <t>user-name@gmail.com</t>
+  </si>
+  <si>
+    <t>test-user@domain.com</t>
+  </si>
+  <si>
+    <t>first-name@company.org</t>
+  </si>
+  <si>
+    <t>abc+test@gmail.com</t>
+  </si>
+  <si>
+    <t>user+1@domain.com</t>
+  </si>
+  <si>
+    <t>firstname+lastname@company.org</t>
+  </si>
+  <si>
+    <t>user.name_123@gmail.com</t>
+  </si>
+  <si>
+    <t>test-user_99@domain.co.in</t>
+  </si>
+  <si>
+    <t>abc.def-123@company.org</t>
+  </si>
+  <si>
+    <t>user@mail.domain.com</t>
+  </si>
+  <si>
+    <t>test@sub.company.org</t>
+  </si>
+  <si>
+    <t>abc@support.google.com</t>
+  </si>
+  <si>
+    <t>user@gmail.co.in</t>
+  </si>
+  <si>
+    <t>test@yahoo.co.uk</t>
+  </si>
+  <si>
+    <t>abc@company.org.in</t>
+  </si>
+  <si>
+    <t>user@domain.co</t>
+  </si>
+  <si>
+    <t>ABC@gmail.com</t>
+  </si>
+  <si>
+    <t>User@Domain.com</t>
+  </si>
+  <si>
+    <t>TEST@YAHOO.COM</t>
+  </si>
+  <si>
+    <t>user@domain.com</t>
+  </si>
+  <si>
+    <t>verylongemailaddress123@gmail.com</t>
+  </si>
+  <si>
+    <t>firstname.lastname.department@companydomain.com</t>
+  </si>
+  <si>
+    <t>user1234567890@subdomain.company.co.in</t>
+  </si>
+  <si>
+    <t>a@b.co</t>
+  </si>
+  <si>
+    <t>x@y.in</t>
+  </si>
+  <si>
+    <t>z@a.io</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -657,6 +1294,14 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -683,10 +1328,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -960,7 +1606,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2509,19 +3155,981 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B167"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="51.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
         <v>21</v>
       </c>
     </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>357</v>
+      </c>
+      <c r="B3" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>196</v>
+      </c>
+      <c r="B4" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>197</v>
+      </c>
+      <c r="B5" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>198</v>
+      </c>
+      <c r="B6" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>199</v>
+      </c>
+      <c r="B7" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>200</v>
+      </c>
+      <c r="B8" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>201</v>
+      </c>
+      <c r="B9" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>202</v>
+      </c>
+      <c r="B10" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11">
+        <v>123456</v>
+      </c>
+      <c r="B11" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" t="s">
+        <v>203</v>
+      </c>
+      <c r="B12" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" t="s">
+        <v>204</v>
+      </c>
+      <c r="B13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>205</v>
+      </c>
+      <c r="B14" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" t="s">
+        <v>206</v>
+      </c>
+      <c r="B15" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" t="s">
+        <v>207</v>
+      </c>
+      <c r="B16" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" t="s">
+        <v>208</v>
+      </c>
+      <c r="B17" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" t="s">
+        <v>209</v>
+      </c>
+      <c r="B18" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" t="s">
+        <v>210</v>
+      </c>
+      <c r="B19" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" t="s">
+        <v>211</v>
+      </c>
+      <c r="B20" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" t="s">
+        <v>212</v>
+      </c>
+      <c r="B21" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" t="s">
+        <v>213</v>
+      </c>
+      <c r="B22" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" t="s">
+        <v>214</v>
+      </c>
+      <c r="B23" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" t="s">
+        <v>215</v>
+      </c>
+      <c r="B24" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" t="s">
+        <v>216</v>
+      </c>
+      <c r="B25" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" t="s">
+        <v>217</v>
+      </c>
+      <c r="B26" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" t="s">
+        <v>218</v>
+      </c>
+      <c r="B27" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" t="s">
+        <v>219</v>
+      </c>
+      <c r="B28" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" t="s">
+        <v>220</v>
+      </c>
+      <c r="B29" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" t="s">
+        <v>221</v>
+      </c>
+      <c r="B30" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" t="s">
+        <v>222</v>
+      </c>
+      <c r="B31" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="A32" t="s">
+        <v>223</v>
+      </c>
+      <c r="B32" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
+      <c r="A33" t="s">
+        <v>224</v>
+      </c>
+      <c r="B33" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" t="s">
+        <v>225</v>
+      </c>
+      <c r="B34" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35" t="s">
+        <v>226</v>
+      </c>
+      <c r="B35" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" t="s">
+        <v>227</v>
+      </c>
+      <c r="B36" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2">
+      <c r="A37" t="s">
+        <v>228</v>
+      </c>
+      <c r="B37" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2">
+      <c r="A38" t="s">
+        <v>229</v>
+      </c>
+      <c r="B38" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2">
+      <c r="A39" t="s">
+        <v>230</v>
+      </c>
+      <c r="B39" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2">
+      <c r="A40" t="s">
+        <v>231</v>
+      </c>
+      <c r="B40" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2">
+      <c r="A41" t="s">
+        <v>232</v>
+      </c>
+      <c r="B41" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2">
+      <c r="A42" t="s">
+        <v>233</v>
+      </c>
+      <c r="B42" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2">
+      <c r="A43" t="s">
+        <v>234</v>
+      </c>
+      <c r="B43" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2">
+      <c r="A44" t="s">
+        <v>235</v>
+      </c>
+      <c r="B44" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2">
+      <c r="A45" t="s">
+        <v>236</v>
+      </c>
+      <c r="B45" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2">
+      <c r="A46" t="s">
+        <v>237</v>
+      </c>
+      <c r="B46" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2">
+      <c r="A47" t="s">
+        <v>238</v>
+      </c>
+      <c r="B47" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2">
+      <c r="A48" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1">
+      <c r="A49" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1">
+      <c r="A50" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1">
+      <c r="A51" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1">
+      <c r="A52" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1">
+      <c r="A53" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1">
+      <c r="A54" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1">
+      <c r="A55" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1">
+      <c r="A56" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1">
+      <c r="A57" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1">
+      <c r="A58" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1">
+      <c r="A59" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1">
+      <c r="A60" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1">
+      <c r="A61" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1">
+      <c r="A62" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1">
+      <c r="A63" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1">
+      <c r="A64" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1">
+      <c r="A65" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1">
+      <c r="A66" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1">
+      <c r="A67" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1">
+      <c r="A68" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1">
+      <c r="A69" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1">
+      <c r="A70" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1">
+      <c r="A71" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1">
+      <c r="A72" s="3" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1">
+      <c r="A73" s="3" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1">
+      <c r="A74" s="3" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1">
+      <c r="A75" s="3" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1">
+      <c r="A76" s="3" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1">
+      <c r="A77" s="3" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1">
+      <c r="A78" s="3" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1">
+      <c r="A79" s="3" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1">
+      <c r="A80" s="3" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1">
+      <c r="A81" s="3" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1">
+      <c r="A82" s="3" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1">
+      <c r="A83" s="3" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1">
+      <c r="A84" s="3" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1">
+      <c r="A85" s="3" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1">
+      <c r="A86" s="3" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1">
+      <c r="A87" s="3" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1">
+      <c r="A88" s="3" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1">
+      <c r="A89" s="3" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1">
+      <c r="A90" s="3" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1">
+      <c r="A91" s="3" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1">
+      <c r="A92" s="3" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1">
+      <c r="A93" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1">
+      <c r="A94" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1">
+      <c r="A95" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1">
+      <c r="A96" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1">
+      <c r="A97" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1">
+      <c r="A98" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1">
+      <c r="A99" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1">
+      <c r="A100" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1">
+      <c r="A101" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1">
+      <c r="A102" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1">
+      <c r="A103" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1">
+      <c r="A104" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1">
+      <c r="A105" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1">
+      <c r="A106" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1">
+      <c r="A107" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1">
+      <c r="A108" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1">
+      <c r="A109" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1">
+      <c r="A110" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1">
+      <c r="A111" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1">
+      <c r="A112" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1">
+      <c r="A113" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1">
+      <c r="A114" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1">
+      <c r="A115" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="116" spans="1:1">
+      <c r="A116" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1">
+      <c r="A117" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1">
+      <c r="A118" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1">
+      <c r="A119" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1">
+      <c r="A120" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1">
+      <c r="A121" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1">
+      <c r="A122" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="123" spans="1:1">
+      <c r="A123" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1">
+      <c r="A124" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="125" spans="1:1">
+      <c r="A125" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1">
+      <c r="A126" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="127" spans="1:1">
+      <c r="A127" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="128" spans="1:1">
+      <c r="A128" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="129" spans="1:1">
+      <c r="A129" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="130" spans="1:1">
+      <c r="A130" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="131" spans="1:1">
+      <c r="A131" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="132" spans="1:1">
+      <c r="A132" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="133" spans="1:1">
+      <c r="A133" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="134" spans="1:1">
+      <c r="A134" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="135" spans="1:1">
+      <c r="A135" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="136" spans="1:1">
+      <c r="A136" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="137" spans="1:1">
+      <c r="A137" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="138" spans="1:1">
+      <c r="A138" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="139" spans="1:1">
+      <c r="A139" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="140" spans="1:1">
+      <c r="A140" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="141" spans="1:1">
+      <c r="A141" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="142" spans="1:1">
+      <c r="A142" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="143" spans="1:1">
+      <c r="A143" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="144" spans="1:1">
+      <c r="A144" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="145" spans="1:1">
+      <c r="A145" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="146" spans="1:1">
+      <c r="A146" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="147" spans="1:1">
+      <c r="A147" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="148" spans="1:1">
+      <c r="A148" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="149" spans="1:1">
+      <c r="A149" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="150" spans="1:1">
+      <c r="A150" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="151" spans="1:1">
+      <c r="A151" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="152" spans="1:1">
+      <c r="A152" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="153" spans="1:1">
+      <c r="A153" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="154" spans="1:1">
+      <c r="A154" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="155" spans="1:1">
+      <c r="A155" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="156" spans="1:1">
+      <c r="A156" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="157" spans="1:1">
+      <c r="A157" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="158" spans="1:1">
+      <c r="A158" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="159" spans="1:1">
+      <c r="A159" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="160" spans="1:1">
+      <c r="A160" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="161" spans="1:1">
+      <c r="A161" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="162" spans="1:1">
+      <c r="A162" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="163" spans="1:1">
+      <c r="A163" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="164" spans="1:1">
+      <c r="A164" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="165" spans="1:1">
+      <c r="A165" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="166" spans="1:1">
+      <c r="A166" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="167" spans="1:1">
+      <c r="A167" t="s">
+        <v>356</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
products page scripts completed
</commit_message>
<xml_diff>
--- a/ecommerse_automation_maven_gurupreeth/project_documents.xlsx
+++ b/ecommerse_automation_maven_gurupreeth/project_documents.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="6" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="916" activeTab="2"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="916" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Homepage" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="400">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="416">
   <si>
     <t>title</t>
   </si>
@@ -1276,6 +1276,54 @@
   </si>
   <si>
     <t>z@a.io</t>
+  </si>
+  <si>
+    <t>NoiseCancel Pro Headphones</t>
+  </si>
+  <si>
+    <t>PulseTrack Fitness Smart Watch</t>
+  </si>
+  <si>
+    <t>Bose QuietComfort Ultra</t>
+  </si>
+  <si>
+    <t>electronics category products</t>
+  </si>
+  <si>
+    <t>Smartphone X1 Pro</t>
+  </si>
+  <si>
+    <t>UltraBook Slim 15</t>
+  </si>
+  <si>
+    <t>Apple iPhone 15 Pro 128GB</t>
+  </si>
+  <si>
+    <t>Samsung Galaxy S24 Ultra</t>
+  </si>
+  <si>
+    <t>OnePlus 12 5G</t>
+  </si>
+  <si>
+    <t>Sony WH-1000XM5</t>
+  </si>
+  <si>
+    <t>Apple MacBook Air M2 13-inch</t>
+  </si>
+  <si>
+    <t>Dell XPS 13 Plus</t>
+  </si>
+  <si>
+    <t>HP Spectre x360 14</t>
+  </si>
+  <si>
+    <t>Apple Watch Series 9 41mm GPS</t>
+  </si>
+  <si>
+    <t>Amazfit GTR 4 Smart Watch</t>
+  </si>
+  <si>
+    <t>Samsung Galaxy Watch6 44mm Bluetooth</t>
   </si>
 </sst>
 </file>
@@ -1606,7 +1654,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -4168,50 +4216,119 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="6" spans="1:1">
+      <c r="B4" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
       <c r="A6" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="7" spans="1:1">
+      <c r="B6" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
       <c r="A7" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="8" spans="1:1">
+      <c r="B7" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
       <c r="A8" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="9" spans="1:1">
+      <c r="B8" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
       <c r="A9" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="10" spans="1:1">
+      <c r="B9" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
       <c r="A10" t="s">
         <v>56</v>
+      </c>
+      <c r="B10" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="B11" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="B12" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="B13" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="B14" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="B15" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="B16" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2">
+      <c r="B17" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2">
+      <c r="B18" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2">
+      <c r="B19" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2">
+      <c r="B20" t="s">
+        <v>414</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updates and new projects
</commit_message>
<xml_diff>
--- a/ecommerse_automation_maven_gurupreeth/project_documents.xlsx
+++ b/ecommerse_automation_maven_gurupreeth/project_documents.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="6" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\eclipse_coding_projects\selenium_automation\ecommerse_automation_maven_gurupreeth\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7A75F25-DB92-4009-A0F4-EDD3A669C0DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="916" activeTab="2"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="916" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Homepage" sheetId="1" r:id="rId1"/>
@@ -33,25 +39,16 @@
     <sheet name="UpdateProfilePage" sheetId="23" r:id="rId24"/>
   </sheets>
   <calcPr calcId="124519"/>
-  <extLst xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main">
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="462">
   <si>
     <t>title</t>
   </si>
@@ -1325,12 +1322,150 @@
   <si>
     <t>Samsung Galaxy Watch6 44mm Bluetooth</t>
   </si>
+  <si>
+    <t>first name input values</t>
+  </si>
+  <si>
+    <t>last name</t>
+  </si>
+  <si>
+    <t>phone</t>
+  </si>
+  <si>
+    <t>message</t>
+  </si>
+  <si>
+    <t xml:space="preserve">valid email ids </t>
+  </si>
+  <si>
+    <t>John</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Jo</t>
+  </si>
+  <si>
+    <t>VeryLongFirstNameExceedingLimit</t>
+  </si>
+  <si>
+    <t>john</t>
+  </si>
+  <si>
+    <t>JOHN</t>
+  </si>
+  <si>
+    <t>JoHn</t>
+  </si>
+  <si>
+    <t>" John"</t>
+  </si>
+  <si>
+    <t>"John "</t>
+  </si>
+  <si>
+    <t>" "</t>
+  </si>
+  <si>
+    <t>""</t>
+  </si>
+  <si>
+    <t>Mary Jane</t>
+  </si>
+  <si>
+    <t>Anne-Marie</t>
+  </si>
+  <si>
+    <t>O'Neil</t>
+  </si>
+  <si>
+    <t>A.J.</t>
+  </si>
+  <si>
+    <t>José</t>
+  </si>
+  <si>
+    <t>राज</t>
+  </si>
+  <si>
+    <t>John1</t>
+  </si>
+  <si>
+    <t>1John</t>
+  </si>
+  <si>
+    <t>Jo1hn</t>
+  </si>
+  <si>
+    <t>@John</t>
+  </si>
+  <si>
+    <t>John@</t>
+  </si>
+  <si>
+    <t>Jo@hn</t>
+  </si>
+  <si>
+    <t>@#$%</t>
+  </si>
+  <si>
+    <t>😀</t>
+  </si>
+  <si>
+    <t>John😀</t>
+  </si>
+  <si>
+    <t>&lt;b&gt;John&lt;/b&gt;</t>
+  </si>
+  <si>
+    <t>&lt;script&gt;alert(1)&lt;/script&gt;</t>
+  </si>
+  <si>
+    <t>' OR '1'='1</t>
+  </si>
+  <si>
+    <t>john@gmail.com</t>
+  </si>
+  <si>
+    <t>https://google.com</t>
+  </si>
+  <si>
+    <t>John_Doe</t>
+  </si>
+  <si>
+    <t>John/Smith</t>
+  </si>
+  <si>
+    <t>John\Smith</t>
+  </si>
+  <si>
+    <t>John\nSmith</t>
+  </si>
+  <si>
+    <t>John\tSmith</t>
+  </si>
+  <si>
+    <t>{"name":"John"}</t>
+  </si>
+  <si>
+    <t>My name is John</t>
+  </si>
+  <si>
+    <t>John,</t>
+  </si>
+  <si>
+    <t>"John"</t>
+  </si>
+  <si>
+    <t>John;</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1654,16 +1789,16 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K123"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.7109375" bestFit="1" customWidth="1"/>
@@ -1677,7 +1812,7 @@
     <col min="10" max="10" width="58.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1694,7 +1829,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1729,12 +1864,12 @@
         <v>66</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D4" s="2">
         <v>49290</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>67</v>
       </c>
@@ -1742,7 +1877,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1</v>
       </c>
@@ -1753,7 +1888,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2</v>
       </c>
@@ -1764,7 +1899,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>3</v>
       </c>
@@ -1775,7 +1910,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>4</v>
       </c>
@@ -1786,7 +1921,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>5</v>
       </c>
@@ -1797,7 +1932,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>6</v>
       </c>
@@ -1808,7 +1943,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>7</v>
       </c>
@@ -1819,7 +1954,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>8</v>
       </c>
@@ -1830,7 +1965,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>9</v>
       </c>
@@ -1841,7 +1976,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>10</v>
       </c>
@@ -1852,7 +1987,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>11</v>
       </c>
@@ -1860,7 +1995,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>12</v>
       </c>
@@ -1868,7 +2003,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>13</v>
       </c>
@@ -1876,7 +2011,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="20" spans="1:2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>14</v>
       </c>
@@ -1884,7 +2019,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>15</v>
       </c>
@@ -1892,7 +2027,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>16</v>
       </c>
@@ -1900,7 +2035,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>17</v>
       </c>
@@ -1908,7 +2043,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="24" spans="1:2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>18</v>
       </c>
@@ -1916,7 +2051,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="25" spans="1:2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>19</v>
       </c>
@@ -1924,7 +2059,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="26" spans="1:2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>20</v>
       </c>
@@ -1932,7 +2067,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="27" spans="1:2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>21</v>
       </c>
@@ -1940,7 +2075,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="28" spans="1:2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>22</v>
       </c>
@@ -1948,7 +2083,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="29" spans="1:2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>23</v>
       </c>
@@ -1956,7 +2091,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="30" spans="1:2">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>24</v>
       </c>
@@ -1964,7 +2099,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="31" spans="1:2">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>25</v>
       </c>
@@ -1972,7 +2107,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="32" spans="1:2">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>26</v>
       </c>
@@ -1980,7 +2115,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="33" spans="1:2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>27</v>
       </c>
@@ -1988,7 +2123,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="34" spans="1:2">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>28</v>
       </c>
@@ -1996,7 +2131,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="35" spans="1:2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>29</v>
       </c>
@@ -2004,7 +2139,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="36" spans="1:2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>30</v>
       </c>
@@ -2012,7 +2147,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="37" spans="1:2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>31</v>
       </c>
@@ -2020,7 +2155,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="38" spans="1:2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>32</v>
       </c>
@@ -2028,7 +2163,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="39" spans="1:2">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>33</v>
       </c>
@@ -2036,7 +2171,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="40" spans="1:2">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>34</v>
       </c>
@@ -2044,7 +2179,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="41" spans="1:2">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>35</v>
       </c>
@@ -2052,7 +2187,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="42" spans="1:2">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>36</v>
       </c>
@@ -2060,7 +2195,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="43" spans="1:2">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>37</v>
       </c>
@@ -2068,7 +2203,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="44" spans="1:2">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>38</v>
       </c>
@@ -2076,7 +2211,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="45" spans="1:2">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>39</v>
       </c>
@@ -2084,7 +2219,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="46" spans="1:2">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>40</v>
       </c>
@@ -2092,7 +2227,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="47" spans="1:2">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>41</v>
       </c>
@@ -2100,7 +2235,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="48" spans="1:2">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>42</v>
       </c>
@@ -2108,7 +2243,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="49" spans="1:2">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>43</v>
       </c>
@@ -2116,7 +2251,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="50" spans="1:2">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>44</v>
       </c>
@@ -2124,7 +2259,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="51" spans="1:2">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>45</v>
       </c>
@@ -2132,7 +2267,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="52" spans="1:2">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>46</v>
       </c>
@@ -2140,7 +2275,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="53" spans="1:2">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>47</v>
       </c>
@@ -2148,7 +2283,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="54" spans="1:2">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>48</v>
       </c>
@@ -2156,7 +2291,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="55" spans="1:2">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>49</v>
       </c>
@@ -2164,7 +2299,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="56" spans="1:2">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>50</v>
       </c>
@@ -2172,7 +2307,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="57" spans="1:2">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>51</v>
       </c>
@@ -2180,7 +2315,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="58" spans="1:2">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>52</v>
       </c>
@@ -2188,7 +2323,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="59" spans="1:2">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>53</v>
       </c>
@@ -2196,7 +2331,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="60" spans="1:2">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>54</v>
       </c>
@@ -2204,7 +2339,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="61" spans="1:2">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>55</v>
       </c>
@@ -2212,7 +2347,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="62" spans="1:2">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>56</v>
       </c>
@@ -2220,7 +2355,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="63" spans="1:2">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>57</v>
       </c>
@@ -2228,7 +2363,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="64" spans="1:2">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>58</v>
       </c>
@@ -2236,7 +2371,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="65" spans="1:2">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>59</v>
       </c>
@@ -2244,7 +2379,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="66" spans="1:2">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>60</v>
       </c>
@@ -2252,7 +2387,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="67" spans="1:2">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>61</v>
       </c>
@@ -2260,7 +2395,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="68" spans="1:2">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>62</v>
       </c>
@@ -2268,7 +2403,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="69" spans="1:2">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>63</v>
       </c>
@@ -2276,7 +2411,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="70" spans="1:2">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>64</v>
       </c>
@@ -2284,7 +2419,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="71" spans="1:2">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>65</v>
       </c>
@@ -2292,7 +2427,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="72" spans="1:2">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>66</v>
       </c>
@@ -2300,7 +2435,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="73" spans="1:2">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>67</v>
       </c>
@@ -2308,7 +2443,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="74" spans="1:2">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>68</v>
       </c>
@@ -2316,7 +2451,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="75" spans="1:2">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>69</v>
       </c>
@@ -2324,7 +2459,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="76" spans="1:2">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>70</v>
       </c>
@@ -2332,7 +2467,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="77" spans="1:2">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>71</v>
       </c>
@@ -2340,7 +2475,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="78" spans="1:2">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>72</v>
       </c>
@@ -2348,7 +2483,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="79" spans="1:2">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>73</v>
       </c>
@@ -2356,7 +2491,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="80" spans="1:2">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>74</v>
       </c>
@@ -2364,7 +2499,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="81" spans="1:2">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>75</v>
       </c>
@@ -2372,7 +2507,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="82" spans="1:2">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>76</v>
       </c>
@@ -2380,7 +2515,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="83" spans="1:2">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>77</v>
       </c>
@@ -2388,7 +2523,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="84" spans="1:2">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>78</v>
       </c>
@@ -2396,7 +2531,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="85" spans="1:2">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>79</v>
       </c>
@@ -2404,7 +2539,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="86" spans="1:2">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>80</v>
       </c>
@@ -2412,7 +2547,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="87" spans="1:2">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>81</v>
       </c>
@@ -2420,7 +2555,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="88" spans="1:2">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>82</v>
       </c>
@@ -2428,7 +2563,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="89" spans="1:2">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>83</v>
       </c>
@@ -2436,7 +2571,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="90" spans="1:2">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>84</v>
       </c>
@@ -2444,7 +2579,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="91" spans="1:2">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>85</v>
       </c>
@@ -2452,7 +2587,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="92" spans="1:2">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>86</v>
       </c>
@@ -2460,7 +2595,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="93" spans="1:2">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>87</v>
       </c>
@@ -2468,7 +2603,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="94" spans="1:2">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>88</v>
       </c>
@@ -2476,7 +2611,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="95" spans="1:2">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>89</v>
       </c>
@@ -2484,7 +2619,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="96" spans="1:2">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>90</v>
       </c>
@@ -2492,7 +2627,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="97" spans="1:2">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>91</v>
       </c>
@@ -2500,7 +2635,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="98" spans="1:2">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>92</v>
       </c>
@@ -2508,7 +2643,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="99" spans="1:2">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>93</v>
       </c>
@@ -2516,7 +2651,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="100" spans="1:2">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>94</v>
       </c>
@@ -2524,7 +2659,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="101" spans="1:2">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>95</v>
       </c>
@@ -2532,7 +2667,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="102" spans="1:2">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>96</v>
       </c>
@@ -2540,7 +2675,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="103" spans="1:2">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>97</v>
       </c>
@@ -2548,7 +2683,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="104" spans="1:2">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>98</v>
       </c>
@@ -2556,7 +2691,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="105" spans="1:2">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>99</v>
       </c>
@@ -2564,7 +2699,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="106" spans="1:2">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>100</v>
       </c>
@@ -2572,7 +2707,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="107" spans="1:2">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>101</v>
       </c>
@@ -2580,7 +2715,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="108" spans="1:2">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>102</v>
       </c>
@@ -2588,7 +2723,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="109" spans="1:2">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>103</v>
       </c>
@@ -2596,7 +2731,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="110" spans="1:2">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>104</v>
       </c>
@@ -2604,7 +2739,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="111" spans="1:2">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>105</v>
       </c>
@@ -2612,7 +2747,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="112" spans="1:2">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>106</v>
       </c>
@@ -2620,7 +2755,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="113" spans="1:2">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>107</v>
       </c>
@@ -2628,7 +2763,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="114" spans="1:2">
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>108</v>
       </c>
@@ -2636,7 +2771,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="115" spans="1:2">
+    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>109</v>
       </c>
@@ -2644,7 +2779,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="116" spans="1:2">
+    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>110</v>
       </c>
@@ -2652,7 +2787,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="117" spans="1:2">
+    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>111</v>
       </c>
@@ -2660,7 +2795,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="118" spans="1:2">
+    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>112</v>
       </c>
@@ -2668,7 +2803,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="119" spans="1:2">
+    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>113</v>
       </c>
@@ -2676,7 +2811,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="120" spans="1:2">
+    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>114</v>
       </c>
@@ -2684,7 +2819,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="121" spans="1:2">
+    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>115</v>
       </c>
@@ -2692,7 +2827,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="122" spans="1:2">
+    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>116</v>
       </c>
@@ -2700,7 +2835,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="123" spans="1:2">
+    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>117</v>
       </c>
@@ -2710,8 +2845,8 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1"/>
-    <hyperlink ref="D2" r:id="rId2"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="D2" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId3"/>
@@ -2719,15 +2854,18 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+  <dimension ref="A1:E214"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="32.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="51.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -2735,7 +2873,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>20</v>
       </c>
@@ -2743,21 +2881,1222 @@
         <v>19</v>
       </c>
     </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>416</v>
+      </c>
+      <c r="B4" t="s">
+        <v>417</v>
+      </c>
+      <c r="C4" t="s">
+        <v>203</v>
+      </c>
+      <c r="D4" t="s">
+        <v>418</v>
+      </c>
+      <c r="E4" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>421</v>
+      </c>
+      <c r="C5" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>422</v>
+      </c>
+      <c r="C6" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>423</v>
+      </c>
+      <c r="C7" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>424</v>
+      </c>
+      <c r="C8" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>425</v>
+      </c>
+      <c r="C9" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>426</v>
+      </c>
+      <c r="C10" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>427</v>
+      </c>
+      <c r="C11" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>428</v>
+      </c>
+      <c r="C12">
+        <v>123456</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>429</v>
+      </c>
+      <c r="C13" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>430</v>
+      </c>
+      <c r="C14" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>431</v>
+      </c>
+      <c r="C15" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>432</v>
+      </c>
+      <c r="C16" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>432</v>
+      </c>
+      <c r="C17" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>433</v>
+      </c>
+      <c r="C18" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>434</v>
+      </c>
+      <c r="C19" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>435</v>
+      </c>
+      <c r="C20" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>436</v>
+      </c>
+      <c r="C21" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>437</v>
+      </c>
+      <c r="C22" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>438</v>
+      </c>
+      <c r="C23" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>439</v>
+      </c>
+      <c r="C24" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>440</v>
+      </c>
+      <c r="C25" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>12345</v>
+      </c>
+      <c r="C26" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>441</v>
+      </c>
+      <c r="C27" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>442</v>
+      </c>
+      <c r="C28" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>443</v>
+      </c>
+      <c r="C29" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>444</v>
+      </c>
+      <c r="C30" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>445</v>
+      </c>
+      <c r="C31" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>446</v>
+      </c>
+      <c r="C32" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>447</v>
+      </c>
+      <c r="C33" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>448</v>
+      </c>
+      <c r="C34" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>449</v>
+      </c>
+      <c r="C35" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>450</v>
+      </c>
+      <c r="C36" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>919876543210</v>
+      </c>
+      <c r="C37" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C38" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>452</v>
+      </c>
+      <c r="C39" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>453</v>
+      </c>
+      <c r="C40" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>454</v>
+      </c>
+      <c r="C41" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>455</v>
+      </c>
+      <c r="C42" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>456</v>
+      </c>
+      <c r="C43" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>457</v>
+      </c>
+      <c r="C44" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>458</v>
+      </c>
+      <c r="C45" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>459</v>
+      </c>
+      <c r="C46" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>460</v>
+      </c>
+      <c r="C47" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>461</v>
+      </c>
+      <c r="C48" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>421</v>
+      </c>
+      <c r="C49" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C50" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C51" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C52" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C53" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C54" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C55" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C56" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C57" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C58" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C59" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C60" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C61" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C62" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C63" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C64" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="65" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C65" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="66" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C66" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="67" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C67" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="68" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C68" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="69" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C69" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="70" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C70" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="71" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C71" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="72" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C72" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="73" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C73" s="3" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="74" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C74" s="3" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="75" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C75" s="3" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="76" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C76" s="3" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="77" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C77" s="3" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="78" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C78" s="3" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="79" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C79" s="3" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="80" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C80" s="3" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="81" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C81" s="3" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="82" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C82" s="3" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="83" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C83" s="3" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="84" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C84" s="3" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="85" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C85" s="3" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="86" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C86" s="3" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="87" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C87" s="3" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="88" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C88" s="3" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="89" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C89" s="3" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="90" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C90" s="3" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="91" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C91" s="3" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="92" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C92" s="3" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="93" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C93" s="3" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="94" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C94" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="95" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C95" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="96" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C96" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="97" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C97" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="98" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C98" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="99" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C99" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="100" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C100" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="101" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C101" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="102" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C102" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="103" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C103" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="104" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C104" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="105" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C105" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="106" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C106" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="107" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C107" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="108" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C108" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="109" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C109" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="110" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C110" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="111" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C111" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="112" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C112" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="113" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C113" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="114" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C114" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="115" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C115" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="116" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C116" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="117" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C117" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="118" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C118" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="119" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C119" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="120" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C120" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="121" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C121" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="122" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C122" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="123" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C123" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="124" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C124" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="125" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C125" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="126" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C126" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="127" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C127" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="128" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C128" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="129" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C129" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="130" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C130" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="131" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C131" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="132" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C132" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="133" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C133" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="134" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C134" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="135" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C135" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="136" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C136" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="137" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C137" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="138" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C138" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="139" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C139" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="140" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C140" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="141" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C141" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="142" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C142" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="143" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C143" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="144" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C144" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="145" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C145" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="146" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C146" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="147" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C147" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="148" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C148" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="149" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C149" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="150" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C150" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="151" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C151" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="152" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C152" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="153" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C153" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="154" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C154" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="155" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C155" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="156" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C156" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="157" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C157" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="158" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C158" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="159" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C159" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="160" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C160" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="161" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C161" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="162" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C162" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="163" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C163" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="164" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C164" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="165" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C165" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="166" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C166" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="167" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C167" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="168" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C168" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="170" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C170" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="171" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C171" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="172" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C172" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="173" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C173" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="174" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C174" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="175" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C175" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="176" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C176" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="177" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C177" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="178" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C178" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="179" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C179" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="180" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C180" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="181" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C181" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="182" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C182" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="183" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C183" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="184" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C184" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="185" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C185" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="186" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C186" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="187" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C187" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="188" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C188" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="189" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C189" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="190" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C190" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="191" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C191" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="192" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C192" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="193" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C193" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="194" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C194" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="195" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C195" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="196" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C196" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="197" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C197" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="198" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C198" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="199" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C199" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="200" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C200" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="201" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C201" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="202" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C202" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="203" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C203" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="204" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C204" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="205" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C205" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="206" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C206" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="207" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C207" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="208" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C208" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="209" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C209" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="210" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C210" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="211" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C211" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="212" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C212" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="213" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C213" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="214" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C214" t="s">
+        <v>399</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A38" r:id="rId1" display="https://google.com/" xr:uid="{7140E357-8D2E-4A2B-BD64-B45EF95395EC}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="27.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -2765,7 +4104,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>23</v>
       </c>
@@ -2779,15 +4118,15 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -2795,7 +4134,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>25</v>
       </c>
@@ -2809,15 +4148,15 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="33.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -2825,7 +4164,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>32</v>
       </c>
@@ -2839,15 +4178,15 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -2855,7 +4194,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>34</v>
       </c>
@@ -2869,11 +4208,11 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2881,7 +4220,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>47</v>
       </c>
@@ -2895,15 +4234,15 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="97.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -2911,7 +4250,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -2925,15 +4264,15 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -2941,7 +4280,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>30</v>
       </c>
@@ -2955,15 +4294,15 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -2971,7 +4310,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>36</v>
       </c>
@@ -2985,15 +4324,15 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -3001,7 +4340,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>37</v>
       </c>
@@ -3015,14 +4354,14 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>22</v>
       </c>
@@ -3033,15 +4372,15 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="27.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -3049,7 +4388,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>39</v>
       </c>
@@ -3063,15 +4402,15 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1400-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="35.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -3079,7 +4418,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>41</v>
       </c>
@@ -3093,15 +4432,15 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -3109,7 +4448,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>45</v>
       </c>
@@ -3123,15 +4462,15 @@
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1600-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="60.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -3139,7 +4478,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>49</v>
       </c>
@@ -3149,22 +4488,22 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-1600-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1700-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="59.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -3172,7 +4511,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>43</v>
       </c>
@@ -3180,7 +4519,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -3188,7 +4527,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>43</v>
       </c>
@@ -3202,20 +4541,20 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B167"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="51.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>357</v>
       </c>
@@ -3223,7 +4562,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>196</v>
       </c>
@@ -3231,7 +4570,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>197</v>
       </c>
@@ -3239,7 +4578,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>198</v>
       </c>
@@ -3247,7 +4586,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>199</v>
       </c>
@@ -3255,7 +4594,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>200</v>
       </c>
@@ -3263,7 +4602,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>201</v>
       </c>
@@ -3271,7 +4610,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>202</v>
       </c>
@@ -3279,7 +4618,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>123456</v>
       </c>
@@ -3287,7 +4626,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>203</v>
       </c>
@@ -3295,7 +4634,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>204</v>
       </c>
@@ -3303,7 +4642,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>205</v>
       </c>
@@ -3311,7 +4650,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>206</v>
       </c>
@@ -3319,7 +4658,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>207</v>
       </c>
@@ -3327,7 +4666,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>208</v>
       </c>
@@ -3335,7 +4674,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>209</v>
       </c>
@@ -3343,7 +4682,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>210</v>
       </c>
@@ -3351,7 +4690,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="20" spans="1:2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>211</v>
       </c>
@@ -3359,7 +4698,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>212</v>
       </c>
@@ -3367,7 +4706,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>213</v>
       </c>
@@ -3375,7 +4714,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>214</v>
       </c>
@@ -3383,7 +4722,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="24" spans="1:2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>215</v>
       </c>
@@ -3391,7 +4730,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="25" spans="1:2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>216</v>
       </c>
@@ -3399,7 +4738,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="26" spans="1:2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>217</v>
       </c>
@@ -3407,7 +4746,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="27" spans="1:2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>218</v>
       </c>
@@ -3415,7 +4754,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="28" spans="1:2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>219</v>
       </c>
@@ -3423,7 +4762,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="29" spans="1:2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>220</v>
       </c>
@@ -3431,7 +4770,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="30" spans="1:2">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>221</v>
       </c>
@@ -3439,7 +4778,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="31" spans="1:2">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>222</v>
       </c>
@@ -3447,7 +4786,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="32" spans="1:2">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>223</v>
       </c>
@@ -3455,7 +4794,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="33" spans="1:2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>224</v>
       </c>
@@ -3463,7 +4802,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="34" spans="1:2">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>225</v>
       </c>
@@ -3471,7 +4810,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="35" spans="1:2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>226</v>
       </c>
@@ -3479,7 +4818,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="36" spans="1:2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>227</v>
       </c>
@@ -3487,7 +4826,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="37" spans="1:2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>228</v>
       </c>
@@ -3495,7 +4834,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="38" spans="1:2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>229</v>
       </c>
@@ -3503,7 +4842,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="39" spans="1:2">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>230</v>
       </c>
@@ -3511,7 +4850,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="40" spans="1:2">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>231</v>
       </c>
@@ -3519,7 +4858,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="41" spans="1:2">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>232</v>
       </c>
@@ -3527,7 +4866,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="42" spans="1:2">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>233</v>
       </c>
@@ -3535,7 +4874,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="43" spans="1:2">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>234</v>
       </c>
@@ -3543,7 +4882,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="44" spans="1:2">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>235</v>
       </c>
@@ -3551,7 +4890,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="45" spans="1:2">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>236</v>
       </c>
@@ -3559,7 +4898,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="46" spans="1:2">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>237</v>
       </c>
@@ -3567,7 +4906,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="47" spans="1:2">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>238</v>
       </c>
@@ -3575,602 +4914,602 @@
         <v>399</v>
       </c>
     </row>
-    <row r="48" spans="1:2">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="49" spans="1:1">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="50" spans="1:1">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="51" spans="1:1">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="52" spans="1:1">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="53" spans="1:1">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="54" spans="1:1">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="55" spans="1:1">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="56" spans="1:1">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="57" spans="1:1">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="58" spans="1:1">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="59" spans="1:1">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="60" spans="1:1">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="61" spans="1:1">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="62" spans="1:1">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="63" spans="1:1">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="64" spans="1:1">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="65" spans="1:1">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="66" spans="1:1">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="67" spans="1:1">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="68" spans="1:1">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="69" spans="1:1">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="70" spans="1:1">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="71" spans="1:1">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="72" spans="1:1">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="73" spans="1:1">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="74" spans="1:1">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="75" spans="1:1">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="76" spans="1:1">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="77" spans="1:1">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="78" spans="1:1">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" s="3" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="79" spans="1:1">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="80" spans="1:1">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="s">
         <v>269</v>
       </c>
     </row>
-    <row r="81" spans="1:1">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="82" spans="1:1">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="83" spans="1:1">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="84" spans="1:1">
+    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="85" spans="1:1">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="86" spans="1:1">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="87" spans="1:1">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="88" spans="1:1">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="s">
         <v>277</v>
       </c>
     </row>
-    <row r="89" spans="1:1">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="90" spans="1:1">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="91" spans="1:1">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="92" spans="1:1">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A92" s="3" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="93" spans="1:1">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="94" spans="1:1">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="95" spans="1:1">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="96" spans="1:1">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="97" spans="1:1">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="98" spans="1:1">
+    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="99" spans="1:1">
+    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="100" spans="1:1">
+    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="101" spans="1:1">
+    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="102" spans="1:1">
+    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="103" spans="1:1">
+    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="104" spans="1:1">
+    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="105" spans="1:1">
+    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="106" spans="1:1">
+    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="107" spans="1:1">
+    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="108" spans="1:1">
+    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="109" spans="1:1">
+    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="110" spans="1:1">
+    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="111" spans="1:1">
+    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="112" spans="1:1">
+    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="113" spans="1:1">
+    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="114" spans="1:1">
+    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="115" spans="1:1">
+    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="116" spans="1:1">
+    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="117" spans="1:1">
+    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="118" spans="1:1">
+    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="119" spans="1:1">
+    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>308</v>
       </c>
     </row>
-    <row r="120" spans="1:1">
+    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="121" spans="1:1">
+    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="122" spans="1:1">
+    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="123" spans="1:1">
+    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="124" spans="1:1">
+    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="125" spans="1:1">
+    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="126" spans="1:1">
+    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="127" spans="1:1">
+    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>316</v>
       </c>
     </row>
-    <row r="128" spans="1:1">
+    <row r="128" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="129" spans="1:1">
+    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>318</v>
       </c>
     </row>
-    <row r="130" spans="1:1">
+    <row r="130" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="131" spans="1:1">
+    <row r="131" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>320</v>
       </c>
     </row>
-    <row r="132" spans="1:1">
+    <row r="132" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="133" spans="1:1">
+    <row r="133" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="134" spans="1:1">
+    <row r="134" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="135" spans="1:1">
+    <row r="135" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>324</v>
       </c>
     </row>
-    <row r="136" spans="1:1">
+    <row r="136" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>325</v>
       </c>
     </row>
-    <row r="137" spans="1:1">
+    <row r="137" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>326</v>
       </c>
     </row>
-    <row r="138" spans="1:1">
+    <row r="138" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>327</v>
       </c>
     </row>
-    <row r="139" spans="1:1">
+    <row r="139" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="140" spans="1:1">
+    <row r="140" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>329</v>
       </c>
     </row>
-    <row r="141" spans="1:1">
+    <row r="141" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>330</v>
       </c>
     </row>
-    <row r="142" spans="1:1">
+    <row r="142" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>331</v>
       </c>
     </row>
-    <row r="143" spans="1:1">
+    <row r="143" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>332</v>
       </c>
     </row>
-    <row r="144" spans="1:1">
+    <row r="144" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>333</v>
       </c>
     </row>
-    <row r="145" spans="1:1">
+    <row r="145" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="146" spans="1:1">
+    <row r="146" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="147" spans="1:1">
+    <row r="147" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>336</v>
       </c>
     </row>
-    <row r="148" spans="1:1">
+    <row r="148" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="149" spans="1:1">
+    <row r="149" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>338</v>
       </c>
     </row>
-    <row r="150" spans="1:1">
+    <row r="150" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>339</v>
       </c>
     </row>
-    <row r="151" spans="1:1">
+    <row r="151" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>340</v>
       </c>
     </row>
-    <row r="152" spans="1:1">
+    <row r="152" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>341</v>
       </c>
     </row>
-    <row r="153" spans="1:1">
+    <row r="153" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>342</v>
       </c>
     </row>
-    <row r="154" spans="1:1">
+    <row r="154" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="155" spans="1:1">
+    <row r="155" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>344</v>
       </c>
     </row>
-    <row r="156" spans="1:1">
+    <row r="156" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>345</v>
       </c>
     </row>
-    <row r="157" spans="1:1">
+    <row r="157" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>346</v>
       </c>
     </row>
-    <row r="158" spans="1:1">
+    <row r="158" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>347</v>
       </c>
     </row>
-    <row r="159" spans="1:1">
+    <row r="159" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>348</v>
       </c>
     </row>
-    <row r="160" spans="1:1">
+    <row r="160" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>349</v>
       </c>
     </row>
-    <row r="161" spans="1:1">
+    <row r="161" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>350</v>
       </c>
     </row>
-    <row r="162" spans="1:1">
+    <row r="162" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>351</v>
       </c>
     </row>
-    <row r="163" spans="1:1">
+    <row r="163" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="164" spans="1:1">
+    <row r="164" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="165" spans="1:1">
+    <row r="165" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>354</v>
       </c>
     </row>
-    <row r="166" spans="1:1">
+    <row r="166" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>355</v>
       </c>
     </row>
-    <row r="167" spans="1:1">
+    <row r="167" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>356</v>
       </c>
@@ -4182,15 +5521,15 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -4198,7 +5537,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -4208,32 +5547,32 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-0300-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:B20"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="35.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>51</v>
       </c>
@@ -4241,7 +5580,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>52</v>
       </c>
@@ -4249,7 +5588,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>53</v>
       </c>
@@ -4257,7 +5596,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>54</v>
       </c>
@@ -4265,7 +5604,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>55</v>
       </c>
@@ -4273,7 +5612,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>56</v>
       </c>
@@ -4281,52 +5620,52 @@
         <v>406</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>407</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>408</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>409</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>402</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>410</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>411</v>
       </c>
     </row>
-    <row r="17" spans="2:2">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>412</v>
       </c>
     </row>
-    <row r="18" spans="2:2">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>413</v>
       </c>
     </row>
-    <row r="19" spans="2:2">
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>415</v>
       </c>
     </row>
-    <row r="20" spans="2:2">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>414</v>
       </c>
@@ -4337,15 +5676,15 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="27.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -4353,7 +5692,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -4367,15 +5706,15 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.28515625" customWidth="1"/>
     <col min="2" max="2" width="27.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -4383,7 +5722,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -4397,14 +5736,14 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -4412,7 +5751,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -4422,22 +5761,22 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-0700-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -4445,7 +5784,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -4455,7 +5794,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-0800-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>